<commit_message>
feat: enhance TimesheetGenerator with dynamic project summary handling and improved Excel export layout
</commit_message>
<xml_diff>
--- a/Aki_Wiksten_05_2026.xlsx
+++ b/Aki_Wiksten_05_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aki Wiksten\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A922FB-240D-4033-ADAD-790EF5F0DA36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7D2A166-17B5-4361-9E27-DDB9CD8479CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD63AFCF-DB4F-455D-A9DD-DFE91348E1A4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="24">
   <si>
     <t>Day of Month</t>
   </si>
@@ -77,21 +77,9 @@
     <t>AJVW Inc.</t>
   </si>
   <si>
-    <t>Project 2</t>
-  </si>
-  <si>
-    <t>Project 3</t>
-  </si>
-  <si>
     <t>Work time total</t>
   </si>
   <si>
-    <t>Design</t>
-  </si>
-  <si>
-    <t>Sum</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -108,6 +96,21 @@
   </si>
   <si>
     <t>End date</t>
+  </si>
+  <si>
+    <t>Kala</t>
+  </si>
+  <si>
+    <t>AWProject</t>
+  </si>
+  <si>
+    <t>Lankku</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>General</t>
   </si>
 </sst>
 </file>
@@ -115,10 +118,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="170" formatCode="mm\/yyyy"/>
-    <numFmt numFmtId="171" formatCode="hh:mm"/>
-    <numFmt numFmtId="172" formatCode="[hh]:mm"/>
-    <numFmt numFmtId="173" formatCode="d\.m\.yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="mm\/yyyy"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="[hh]:mm"/>
+    <numFmt numFmtId="167" formatCode="d\.m\.yyyy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -252,55 +255,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -635,7 +631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EE29E80-1386-45A8-BD1E-FE65E759F17A}">
-  <dimension ref="A1:AF24"/>
+  <dimension ref="A1:AF23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.1796875" customWidth="1"/>
@@ -643,228 +639,213 @@
     <col min="4" max="4" width="15.453125" customWidth="1"/>
     <col min="7" max="7" width="8.7265625" customWidth="1"/>
     <col min="9" max="9" width="11.08984375" customWidth="1"/>
-    <col min="10" max="10" width="9.81640625" customWidth="1"/>
+    <col min="10" max="11" width="9.81640625" customWidth="1"/>
+    <col min="13" max="13" width="10.90625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="D1" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14" t="s">
+      <c r="H1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="I1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="12"/>
+      <c r="K1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="V1" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="W1" s="13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="E2" s="30">
+        <v>0.22916666666666699</v>
+      </c>
+      <c r="F2" s="30">
+        <v>0.29166666666666702</v>
+      </c>
+      <c r="G2" s="30">
+        <v>0.104166666666667</v>
+      </c>
+      <c r="H2" s="30">
+        <v>0.375</v>
+      </c>
+      <c r="I2" s="20">
+        <v>1</v>
+      </c>
+      <c r="J2" s="28"/>
+      <c r="K2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="L2" s="23">
+        <v>1</v>
+      </c>
+      <c r="M2" s="23">
+        <v>2</v>
+      </c>
+      <c r="N2" s="23">
+        <v>0</v>
+      </c>
+      <c r="O2" s="23">
+        <v>2</v>
+      </c>
+      <c r="P2" s="25">
+        <v>5</v>
+      </c>
+      <c r="R2" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="S2" s="18">
+        <v>0.22916666666666699</v>
+      </c>
+      <c r="T2" s="18">
+        <v>0.29166666666666702</v>
+      </c>
+      <c r="U2" s="18">
+        <v>0.104166666666667</v>
+      </c>
+      <c r="V2" s="18">
+        <v>0.375</v>
+      </c>
+      <c r="W2" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="14">
+        <v>30</v>
+      </c>
+      <c r="F3" s="14">
+        <v>140</v>
+      </c>
+      <c r="G3" s="14">
+        <v>20</v>
+      </c>
+      <c r="H3" s="14">
+        <v>100</v>
+      </c>
+      <c r="I3" s="15">
+        <v>290</v>
+      </c>
+      <c r="J3" s="29"/>
+      <c r="K3" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="23">
+        <v>0</v>
+      </c>
+      <c r="M3" s="23">
+        <v>0</v>
+      </c>
+      <c r="N3" s="23">
+        <v>1</v>
+      </c>
+      <c r="O3" s="23">
+        <v>0</v>
+      </c>
+      <c r="P3" s="25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q1" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="S1" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="T1" s="31" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="16">
-        <f>SUM(B9,G9)</f>
-        <v>0.375</v>
-      </c>
-      <c r="F2" s="16">
-        <f>SUM(B15,E9,G15)</f>
-        <v>0.39583333333333337</v>
-      </c>
-      <c r="G2" s="16">
-        <f>SUM(E15,G21)</f>
-        <v>0.25</v>
-      </c>
-      <c r="H2" s="27">
-        <f>SUM(E2,F2,G2)</f>
-        <v>1.0208333333333335</v>
-      </c>
-      <c r="I2" s="26"/>
-      <c r="J2" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" s="30">
-        <v>1</v>
-      </c>
-      <c r="L2" s="30">
-        <v>1</v>
-      </c>
-      <c r="M2" s="30">
+      <c r="B4" s="21">
+        <v>46143</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="26">
         <v>0</v>
       </c>
-      <c r="N2" s="33">
-        <v>2</v>
-      </c>
-      <c r="P2" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q2" s="16">
-        <f>SUM(B9,G9)</f>
-        <v>0.375</v>
-      </c>
-      <c r="R2" s="16">
-        <f>SUM(B15,E9)</f>
-        <v>0.25</v>
-      </c>
-      <c r="S2" s="16">
-        <f>SUM(G21)</f>
-        <v>0.1875</v>
-      </c>
-      <c r="T2" s="17">
-        <f>SUM(Q2:S2)</f>
-        <v>0.8125</v>
-      </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="19">
-        <f>SUM(B12,G12)</f>
-        <v>140</v>
-      </c>
-      <c r="F3" s="19">
-        <f>SUM(B18,E12,G18)</f>
-        <v>220</v>
-      </c>
-      <c r="G3" s="19">
-        <f>SUM(E18,G24)</f>
-        <v>240</v>
-      </c>
-      <c r="H3" s="20">
-        <f>SUM(E3,F3,G3)</f>
-        <v>600</v>
-      </c>
-      <c r="I3" s="18"/>
-      <c r="J3" s="34" t="s">
+      <c r="M4" s="26">
+        <v>0</v>
+      </c>
+      <c r="N4" s="26">
+        <v>0</v>
+      </c>
+      <c r="O4" s="26">
+        <v>0</v>
+      </c>
+      <c r="P4" s="27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="30">
-        <v>0</v>
-      </c>
-      <c r="L3" s="30">
-        <v>1</v>
-      </c>
-      <c r="M3" s="30">
-        <v>0</v>
-      </c>
-      <c r="N3" s="33">
-        <v>1</v>
-      </c>
-      <c r="P3" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="23">
-        <f>SUM(G15)</f>
-        <v>0.14583333333333334</v>
-      </c>
-      <c r="S3" s="23">
-        <f>SUM(E15)</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="T3" s="24">
-        <f>SUM(Q3:S3)</f>
-        <v>0.20833333333333334</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="28">
-        <v>46143</v>
-      </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="36">
-        <v>1</v>
-      </c>
-      <c r="L4" s="36">
-        <v>1</v>
-      </c>
-      <c r="M4" s="36">
-        <v>2</v>
-      </c>
-      <c r="N4" s="37">
-        <v>4</v>
-      </c>
-      <c r="P4" s="7"/>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="29">
+      <c r="B5" s="22">
         <v>46173</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="O5" s="7"/>
+      <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
@@ -972,16 +953,22 @@
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
-      <c r="E8" s="5" t="s">
-        <v>12</v>
-      </c>
+      <c r="E8" s="5"/>
       <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="5"/>
+      <c r="N8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q8" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -989,44 +976,62 @@
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="6">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="E9" s="6">
+      <c r="B9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="N9" s="6">
+        <v>0.22916666666666699</v>
+      </c>
+      <c r="O9" s="6">
+        <v>0.14583333333333301</v>
+      </c>
+      <c r="P9" s="6">
+        <v>0.14583333333333301</v>
+      </c>
+      <c r="Q9" s="6">
         <v>0.1875</v>
-      </c>
-      <c r="G9" s="6">
-        <v>0.10416666666666667</v>
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="E10" s="5"/>
       <c r="F10" s="5"/>
-      <c r="G10" s="5" t="s">
-        <v>19</v>
+      <c r="G10" s="5"/>
+      <c r="N10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="O10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="N11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="O11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="P11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1034,105 +1039,92 @@
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12">
-        <v>70</v>
-      </c>
-      <c r="E12">
-        <v>40</v>
-      </c>
-      <c r="G12">
-        <v>70</v>
+      <c r="N12">
+        <v>30</v>
+      </c>
+      <c r="O12">
+        <v>80</v>
+      </c>
+      <c r="P12">
+        <v>60</v>
+      </c>
+      <c r="Q12">
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
-      <c r="B14" s="5" t="s">
-        <v>12</v>
-      </c>
+      <c r="B14" s="5"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
-      <c r="E14" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="E14" s="5"/>
       <c r="F14" s="5"/>
-      <c r="G14" s="5" t="s">
-        <v>12</v>
+      <c r="G14" s="5"/>
+      <c r="O14" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="P14" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
-      <c r="B15" s="6">
-        <v>6.25E-2</v>
-      </c>
-      <c r="E15" s="6">
-        <v>6.25E-2</v>
-      </c>
-      <c r="G15" s="6">
-        <v>0.14583333333333334</v>
+      <c r="B15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="O15" s="6">
+        <v>0.104166666666667</v>
+      </c>
+      <c r="P15" s="6">
+        <v>0.1875</v>
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
-      <c r="B16" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="E16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="O16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="P16" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="O17" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="P17" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
-      <c r="B18">
-        <v>90</v>
-      </c>
-      <c r="E18">
-        <v>120</v>
-      </c>
-      <c r="G18">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G20" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G21" s="6">
-        <v>0.1875</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G22" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G23" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G24">
-        <v>120</v>
-      </c>
+      <c r="O18">
+        <v>20</v>
+      </c>
+      <c r="P18">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G20" s="5"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G22" s="5"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="G23" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>